<commit_message>
fourth commit on 30/10
</commit_message>
<xml_diff>
--- a/testData/TestScriptData.xlsx
+++ b/testData/TestScriptData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prath\Desktop\VTiger_Playwright\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A9F616-274F-41BE-BA38-35B5351C8D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78951E27-A832-4E98-8B15-8CC039787A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contacts" sheetId="1" r:id="rId1"/>
+    <sheet name="Organizations" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>First Name</t>
   </si>
@@ -49,6 +50,18 @@
   </si>
   <si>
     <t>Singh</t>
+  </si>
+  <si>
+    <t>Organization_Name</t>
+  </si>
+  <si>
+    <t>TekPyramid</t>
+  </si>
+  <si>
+    <t>TestYantra</t>
+  </si>
+  <si>
+    <t>Qspiders</t>
   </si>
 </sst>
 </file>
@@ -408,4 +421,37 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6F297F1-0C02-4753-9693-52C75178D120}">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>